<commit_message>
Added survey result and clean up Nutzwertanalyse.xlsx
</commit_message>
<xml_diff>
--- a/Nutzwertanalyse_Kategorien.xlsx
+++ b/Nutzwertanalyse_Kategorien.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8a471988a8a86cc1/Studium/Bachelor/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8a471988a8a86cc1/Studium/Bachelor/Artefakte/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="200" documentId="8_{445BECBA-4A71-4BA1-B588-6903AAB647EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8FDFF28C-AEBE-4138-8DA7-04BEBAAE0EA5}"/>
+  <xr:revisionPtr revIDLastSave="214" documentId="8_{445BECBA-4A71-4BA1-B588-6903AAB647EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A50A1BD-1B44-45C4-8E11-9FA808205190}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="8" xr2:uid="{20C679E4-C9D8-48C4-B659-4235CD5DE514}"/>
+    <workbookView xWindow="-28920" yWindow="345" windowWidth="29040" windowHeight="15720" xr2:uid="{20C679E4-C9D8-48C4-B659-4235CD5DE514}"/>
   </bookViews>
   <sheets>
     <sheet name="Szenarien" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="51">
   <si>
     <t>Szenario</t>
   </si>
@@ -194,9 +194,6 @@
     <t>Unified Storage: Objekt</t>
   </si>
   <si>
-    <t>TODO: Werte Prüfen? / Nur die ohne Split</t>
-  </si>
-  <si>
     <t>Verschlüsselung</t>
   </si>
   <si>
@@ -207,9 +204,6 @@
   </si>
   <si>
     <t>Objekt</t>
-  </si>
-  <si>
-    <t>TODO: Neutrales Szenario</t>
   </si>
   <si>
     <t>Storage-Features: Datenlokalität</t>
@@ -225,6 +219,9 @@
   </si>
   <si>
     <t>Storage-Features: Daten-Effizienz</t>
+  </si>
+  <si>
+    <t>#</t>
   </si>
 </sst>
 </file>
@@ -397,7 +394,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -415,43 +412,12 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="12" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -466,6 +432,36 @@
     </xf>
     <xf numFmtId="12" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -809,45 +805,45 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="16" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="16" t="s">
+      <c r="A1" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="14"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="I1" s="14"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="16" t="s">
+      <c r="E1" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="23"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" s="23"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="12" t="s">
+      <c r="L1" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="13" t="s">
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="P1" s="14"/>
-      <c r="Q1" s="15"/>
-      <c r="R1" s="16" t="s">
+      <c r="P1" s="23"/>
+      <c r="Q1" s="24"/>
+      <c r="R1" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="S1" s="16" t="s">
+      <c r="S1" s="17" t="s">
         <v>6</v>
       </c>
       <c r="T1" s="19" t="s">
@@ -858,49 +854,49 @@
       </c>
     </row>
     <row r="2" spans="1:21" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" s="17"/>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="11" t="s">
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="F2" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H2" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="I2" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="J2" s="11" t="s">
+      <c r="J2" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="K2" s="17"/>
-      <c r="L2" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="M2" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="N2" s="11" t="s">
+      <c r="K2" s="18"/>
+      <c r="L2" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="M2" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="N2" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="O2" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="O2" s="11" t="s">
+      <c r="P2" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="P2" s="11" t="s">
+      <c r="Q2" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="Q2" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="R2" s="17"/>
-      <c r="S2" s="17"/>
+      <c r="R2" s="18"/>
+      <c r="S2" s="18"/>
       <c r="T2" s="20"/>
       <c r="U2" s="20"/>
     </row>
@@ -908,65 +904,65 @@
       <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="22">
+      <c r="B3" s="11">
         <v>50</v>
       </c>
-      <c r="C3" s="22">
+      <c r="C3" s="11">
         <v>5</v>
       </c>
-      <c r="D3" s="22">
-        <v>0</v>
-      </c>
-      <c r="E3" s="22">
-        <v>10</v>
-      </c>
-      <c r="F3" s="22">
+      <c r="D3" s="11">
+        <v>0</v>
+      </c>
+      <c r="E3" s="11">
+        <v>10</v>
+      </c>
+      <c r="F3" s="11">
         <v>5</v>
       </c>
-      <c r="G3" s="22">
-        <v>0</v>
-      </c>
-      <c r="H3" s="22">
+      <c r="G3" s="11">
+        <v>0</v>
+      </c>
+      <c r="H3" s="11">
         <v>7</v>
       </c>
-      <c r="I3" s="22">
-        <v>0</v>
-      </c>
-      <c r="J3" s="22">
-        <v>3</v>
-      </c>
-      <c r="K3" s="22">
-        <v>0</v>
-      </c>
-      <c r="L3" s="22">
+      <c r="I3" s="11">
+        <v>0</v>
+      </c>
+      <c r="J3" s="11">
+        <v>3</v>
+      </c>
+      <c r="K3" s="11">
+        <v>0</v>
+      </c>
+      <c r="L3" s="11">
         <v>2.5</v>
       </c>
-      <c r="M3" s="22">
+      <c r="M3" s="11">
         <v>2.5</v>
       </c>
-      <c r="N3" s="22">
-        <v>0</v>
-      </c>
-      <c r="O3" s="22">
-        <v>0</v>
-      </c>
-      <c r="P3" s="22">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="22">
-        <v>0</v>
-      </c>
-      <c r="R3" s="22">
-        <v>10</v>
-      </c>
-      <c r="S3" s="22">
+      <c r="N3" s="11">
+        <v>0</v>
+      </c>
+      <c r="O3" s="11">
+        <v>0</v>
+      </c>
+      <c r="P3" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="11">
+        <v>0</v>
+      </c>
+      <c r="R3" s="11">
+        <v>10</v>
+      </c>
+      <c r="S3" s="11">
         <v>5</v>
       </c>
       <c r="T3" s="3">
         <f t="shared" ref="T3:T8" si="0">SUM(B3:S3)</f>
         <v>100</v>
       </c>
-      <c r="U3" s="9">
+      <c r="U3" s="21">
         <f>AVERAGE(T3:T7)</f>
         <v>100</v>
       </c>
@@ -975,314 +971,314 @@
       <c r="A4" s="6">
         <v>2</v>
       </c>
-      <c r="B4" s="23">
-        <v>15</v>
-      </c>
-      <c r="C4" s="23">
-        <v>10</v>
-      </c>
-      <c r="D4" s="23">
-        <v>15</v>
-      </c>
-      <c r="E4" s="23">
+      <c r="B4" s="12">
+        <v>15</v>
+      </c>
+      <c r="C4" s="12">
+        <v>10</v>
+      </c>
+      <c r="D4" s="12">
+        <v>15</v>
+      </c>
+      <c r="E4" s="12">
         <v>5</v>
       </c>
-      <c r="F4" s="23">
-        <v>0</v>
-      </c>
-      <c r="G4" s="23">
-        <v>0</v>
-      </c>
-      <c r="H4" s="23">
-        <v>15</v>
-      </c>
-      <c r="I4" s="23">
-        <v>0</v>
-      </c>
-      <c r="J4" s="23">
-        <v>0</v>
-      </c>
-      <c r="K4" s="23">
-        <v>15</v>
-      </c>
-      <c r="L4" s="22">
+      <c r="F4" s="12">
+        <v>0</v>
+      </c>
+      <c r="G4" s="12">
+        <v>0</v>
+      </c>
+      <c r="H4" s="12">
+        <v>15</v>
+      </c>
+      <c r="I4" s="12">
+        <v>0</v>
+      </c>
+      <c r="J4" s="12">
+        <v>0</v>
+      </c>
+      <c r="K4" s="12">
+        <v>15</v>
+      </c>
+      <c r="L4" s="11">
         <v>2.5</v>
       </c>
-      <c r="M4" s="22">
+      <c r="M4" s="11">
         <v>2.5</v>
       </c>
-      <c r="N4" s="23">
-        <v>0</v>
-      </c>
-      <c r="O4" s="23">
-        <v>0</v>
-      </c>
-      <c r="P4" s="23">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="23">
-        <v>0</v>
-      </c>
-      <c r="R4" s="23">
-        <v>15</v>
-      </c>
-      <c r="S4" s="23">
+      <c r="N4" s="12">
+        <v>0</v>
+      </c>
+      <c r="O4" s="12">
+        <v>0</v>
+      </c>
+      <c r="P4" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="12">
+        <v>0</v>
+      </c>
+      <c r="R4" s="12">
+        <v>15</v>
+      </c>
+      <c r="S4" s="12">
         <v>5</v>
       </c>
       <c r="T4" s="3">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="U4" s="9"/>
+      <c r="U4" s="21"/>
     </row>
     <row r="5" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6">
         <v>3</v>
       </c>
-      <c r="B5" s="23">
-        <v>15</v>
-      </c>
-      <c r="C5" s="23">
-        <v>10</v>
-      </c>
-      <c r="D5" s="23">
-        <v>15</v>
-      </c>
-      <c r="E5" s="23">
+      <c r="B5" s="12">
+        <v>15</v>
+      </c>
+      <c r="C5" s="12">
+        <v>10</v>
+      </c>
+      <c r="D5" s="12">
+        <v>15</v>
+      </c>
+      <c r="E5" s="12">
         <v>5</v>
       </c>
-      <c r="F5" s="23">
-        <v>0</v>
-      </c>
-      <c r="G5" s="23">
-        <v>0</v>
-      </c>
-      <c r="H5" s="23">
+      <c r="F5" s="12">
+        <v>0</v>
+      </c>
+      <c r="G5" s="12">
+        <v>0</v>
+      </c>
+      <c r="H5" s="12">
         <v>5</v>
       </c>
-      <c r="I5" s="23">
-        <v>0</v>
-      </c>
-      <c r="J5" s="23">
-        <v>0</v>
-      </c>
-      <c r="K5" s="23">
-        <v>0</v>
-      </c>
-      <c r="L5" s="23">
+      <c r="I5" s="12">
+        <v>0</v>
+      </c>
+      <c r="J5" s="12">
+        <v>0</v>
+      </c>
+      <c r="K5" s="12">
+        <v>0</v>
+      </c>
+      <c r="L5" s="12">
         <v>5</v>
       </c>
-      <c r="M5" s="23">
-        <v>10</v>
-      </c>
-      <c r="N5" s="23">
-        <v>0</v>
-      </c>
-      <c r="O5" s="23">
-        <v>0</v>
-      </c>
-      <c r="P5" s="23">
-        <v>10</v>
-      </c>
-      <c r="Q5" s="23">
+      <c r="M5" s="12">
+        <v>10</v>
+      </c>
+      <c r="N5" s="12">
+        <v>0</v>
+      </c>
+      <c r="O5" s="12">
+        <v>0</v>
+      </c>
+      <c r="P5" s="12">
+        <v>10</v>
+      </c>
+      <c r="Q5" s="12">
         <v>5</v>
       </c>
-      <c r="R5" s="23">
-        <v>15</v>
-      </c>
-      <c r="S5" s="23">
+      <c r="R5" s="12">
+        <v>15</v>
+      </c>
+      <c r="S5" s="12">
         <v>5</v>
       </c>
       <c r="T5" s="3">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="U5" s="9"/>
+      <c r="U5" s="21"/>
     </row>
     <row r="6" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="6">
         <v>4</v>
       </c>
-      <c r="B6" s="23">
-        <v>10</v>
-      </c>
-      <c r="C6" s="23">
-        <v>10</v>
-      </c>
-      <c r="D6" s="23">
-        <v>10</v>
-      </c>
-      <c r="E6" s="23">
+      <c r="B6" s="12">
+        <v>10</v>
+      </c>
+      <c r="C6" s="12">
+        <v>10</v>
+      </c>
+      <c r="D6" s="12">
+        <v>10</v>
+      </c>
+      <c r="E6" s="12">
         <v>5</v>
       </c>
-      <c r="F6" s="23">
-        <v>0</v>
-      </c>
-      <c r="G6" s="23">
+      <c r="F6" s="12">
+        <v>0</v>
+      </c>
+      <c r="G6" s="12">
         <v>5</v>
       </c>
-      <c r="H6" s="23">
+      <c r="H6" s="12">
         <v>5</v>
       </c>
-      <c r="I6" s="23">
-        <v>10</v>
-      </c>
-      <c r="J6" s="23">
-        <v>0</v>
-      </c>
-      <c r="K6" s="23">
-        <v>0</v>
-      </c>
-      <c r="L6" s="23">
+      <c r="I6" s="12">
+        <v>10</v>
+      </c>
+      <c r="J6" s="12">
+        <v>0</v>
+      </c>
+      <c r="K6" s="12">
+        <v>0</v>
+      </c>
+      <c r="L6" s="12">
         <v>5</v>
       </c>
-      <c r="M6" s="23">
+      <c r="M6" s="12">
         <v>5</v>
       </c>
-      <c r="N6" s="23">
+      <c r="N6" s="12">
         <v>5</v>
       </c>
-      <c r="O6" s="23">
-        <v>10</v>
-      </c>
-      <c r="P6" s="23">
+      <c r="O6" s="12">
+        <v>10</v>
+      </c>
+      <c r="P6" s="12">
         <v>5</v>
       </c>
-      <c r="Q6" s="23">
-        <v>0</v>
-      </c>
-      <c r="R6" s="23">
-        <v>10</v>
-      </c>
-      <c r="S6" s="23">
+      <c r="Q6" s="12">
+        <v>0</v>
+      </c>
+      <c r="R6" s="12">
+        <v>10</v>
+      </c>
+      <c r="S6" s="12">
         <v>5</v>
       </c>
       <c r="T6" s="3">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="U6" s="9"/>
+      <c r="U6" s="21"/>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="8">
         <v>5</v>
       </c>
-      <c r="B7" s="24">
+      <c r="B7" s="13">
         <v>5</v>
       </c>
-      <c r="C7" s="24">
-        <v>15</v>
-      </c>
-      <c r="D7" s="24">
-        <v>10</v>
-      </c>
-      <c r="E7" s="24">
-        <v>0</v>
-      </c>
-      <c r="F7" s="24">
-        <v>0</v>
-      </c>
-      <c r="G7" s="24">
-        <v>10</v>
-      </c>
-      <c r="H7" s="24">
+      <c r="C7" s="13">
+        <v>15</v>
+      </c>
+      <c r="D7" s="13">
+        <v>10</v>
+      </c>
+      <c r="E7" s="13">
+        <v>0</v>
+      </c>
+      <c r="F7" s="13">
+        <v>0</v>
+      </c>
+      <c r="G7" s="13">
+        <v>10</v>
+      </c>
+      <c r="H7" s="13">
         <v>5</v>
       </c>
-      <c r="I7" s="24">
-        <v>0</v>
-      </c>
-      <c r="J7" s="24">
-        <v>10</v>
-      </c>
-      <c r="K7" s="24">
-        <v>15</v>
-      </c>
-      <c r="L7" s="24">
-        <v>0</v>
-      </c>
-      <c r="M7" s="24">
-        <v>3</v>
-      </c>
-      <c r="N7" s="24">
+      <c r="I7" s="13">
+        <v>0</v>
+      </c>
+      <c r="J7" s="13">
+        <v>10</v>
+      </c>
+      <c r="K7" s="13">
+        <v>15</v>
+      </c>
+      <c r="L7" s="13">
+        <v>0</v>
+      </c>
+      <c r="M7" s="13">
+        <v>3</v>
+      </c>
+      <c r="N7" s="13">
         <v>7</v>
       </c>
-      <c r="O7" s="24">
-        <v>0</v>
-      </c>
-      <c r="P7" s="24">
+      <c r="O7" s="13">
+        <v>0</v>
+      </c>
+      <c r="P7" s="13">
         <v>5</v>
       </c>
-      <c r="Q7" s="24">
-        <v>0</v>
-      </c>
-      <c r="R7" s="24">
+      <c r="Q7" s="13">
+        <v>0</v>
+      </c>
+      <c r="R7" s="13">
         <v>5</v>
       </c>
-      <c r="S7" s="24">
+      <c r="S7" s="13">
         <v>10</v>
       </c>
       <c r="T7" s="3">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="U7" s="9"/>
+      <c r="U7" s="21"/>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="6">
         <v>0</v>
       </c>
-      <c r="B8" s="25">
-        <v>10</v>
-      </c>
-      <c r="C8" s="25">
-        <v>10</v>
-      </c>
-      <c r="D8" s="25">
-        <v>10</v>
-      </c>
-      <c r="E8" s="25">
+      <c r="B8" s="14">
+        <v>10</v>
+      </c>
+      <c r="C8" s="14">
+        <v>10</v>
+      </c>
+      <c r="D8" s="14">
+        <v>10</v>
+      </c>
+      <c r="E8" s="14">
         <v>3.3333333000000001</v>
       </c>
-      <c r="F8" s="25">
+      <c r="F8" s="14">
         <v>3.3333333000000001</v>
       </c>
-      <c r="G8" s="25">
+      <c r="G8" s="14">
         <v>3.3333333000000001</v>
       </c>
-      <c r="H8" s="25">
+      <c r="H8" s="14">
         <v>3.3333333000000001</v>
       </c>
-      <c r="I8" s="25">
+      <c r="I8" s="14">
         <v>3.3333333000000001</v>
       </c>
-      <c r="J8" s="25">
+      <c r="J8" s="14">
         <v>3.3333333000000001</v>
       </c>
-      <c r="K8" s="25">
-        <v>10</v>
-      </c>
-      <c r="L8" s="25">
+      <c r="K8" s="14">
+        <v>10</v>
+      </c>
+      <c r="L8" s="14">
         <v>3.3333333000000001</v>
       </c>
-      <c r="M8" s="25">
+      <c r="M8" s="14">
         <v>3.3333333000000001</v>
       </c>
-      <c r="N8" s="25">
+      <c r="N8" s="14">
         <v>3.3333333000000001</v>
       </c>
-      <c r="O8" s="25">
+      <c r="O8" s="14">
         <v>3.3333333000000001</v>
       </c>
-      <c r="P8" s="25">
+      <c r="P8" s="14">
         <v>3.3333333000000001</v>
       </c>
-      <c r="Q8" s="25">
+      <c r="Q8" s="14">
         <v>3.3333333000000001</v>
       </c>
-      <c r="R8" s="25">
-        <v>10</v>
-      </c>
-      <c r="S8" s="25">
+      <c r="R8" s="14">
+        <v>10</v>
+      </c>
+      <c r="S8" s="14">
         <v>10</v>
       </c>
       <c r="T8" s="3">
@@ -1295,79 +1291,79 @@
       <c r="A9" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="26">
+      <c r="B9" s="15">
         <f t="shared" ref="B9:S9" si="1">SUM(B3:B8)</f>
         <v>105</v>
       </c>
-      <c r="C9" s="26">
+      <c r="C9" s="15">
         <f t="shared" si="1"/>
         <v>60</v>
       </c>
-      <c r="D9" s="26">
+      <c r="D9" s="15">
         <f t="shared" si="1"/>
         <v>60</v>
       </c>
-      <c r="E9" s="26">
+      <c r="E9" s="15">
         <f t="shared" si="1"/>
         <v>28.3333333</v>
       </c>
-      <c r="F9" s="26">
+      <c r="F9" s="15">
         <f t="shared" ref="F9" si="2">SUM(F3:F8)</f>
         <v>8.3333332999999996</v>
       </c>
-      <c r="G9" s="26">
+      <c r="G9" s="15">
         <f t="shared" ref="G9" si="3">SUM(G3:G8)</f>
         <v>18.3333333</v>
       </c>
-      <c r="H9" s="26">
+      <c r="H9" s="15">
         <f t="shared" ref="H9" si="4">SUM(H3:H8)</f>
         <v>40.3333333</v>
       </c>
-      <c r="I9" s="26">
+      <c r="I9" s="15">
         <f t="shared" ref="I9" si="5">SUM(I3:I8)</f>
         <v>13.3333333</v>
       </c>
-      <c r="J9" s="26">
+      <c r="J9" s="15">
         <f t="shared" ref="J9" si="6">SUM(J3:J8)</f>
         <v>16.3333333</v>
       </c>
-      <c r="K9" s="26">
+      <c r="K9" s="15">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="L9" s="26">
+      <c r="L9" s="15">
         <f t="shared" si="1"/>
         <v>18.3333333</v>
       </c>
-      <c r="M9" s="26">
+      <c r="M9" s="15">
         <f t="shared" ref="M9" si="7">SUM(M3:M8)</f>
         <v>26.3333333</v>
       </c>
-      <c r="N9" s="26">
+      <c r="N9" s="15">
         <f t="shared" ref="N9" si="8">SUM(N3:N8)</f>
         <v>15.3333333</v>
       </c>
-      <c r="O9" s="26">
+      <c r="O9" s="15">
         <f t="shared" si="1"/>
         <v>13.3333333</v>
       </c>
-      <c r="P9" s="26">
+      <c r="P9" s="15">
         <f t="shared" ref="P9" si="9">SUM(P3:P8)</f>
         <v>23.3333333</v>
       </c>
-      <c r="Q9" s="26">
+      <c r="Q9" s="15">
         <f t="shared" ref="Q9" si="10">SUM(Q3:Q8)</f>
         <v>8.3333332999999996</v>
       </c>
-      <c r="R9" s="26">
+      <c r="R9" s="15">
         <f t="shared" si="1"/>
         <v>65</v>
       </c>
-      <c r="S9" s="26">
+      <c r="S9" s="15">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="T9" s="18" t="s">
+      <c r="T9" s="10" t="s">
         <v>20</v>
       </c>
       <c r="U9" s="3">
@@ -1377,11 +1373,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="O1:Q1"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="B1:B2"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="T1:T2"/>
     <mergeCell ref="U3:U7"/>
@@ -1391,6 +1382,11 @@
     <mergeCell ref="R1:R2"/>
     <mergeCell ref="S1:S2"/>
     <mergeCell ref="U1:U2"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="O1:Q1"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="B1:B2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1425,10 +1421,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" s="2">
         <v>3</v>
@@ -1562,7 +1558,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B12" s="2">
         <v>3</v>
@@ -1576,7 +1572,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B13" s="2">
         <v>3</v>
@@ -1678,11 +1674,11 @@
       </c>
       <c r="B20" s="5">
         <f>SUM(B2:B19)</f>
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C20" s="5">
         <f t="shared" ref="C20:D20" si="0">SUM(C2:C19)</f>
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D20" s="5">
         <f t="shared" si="0"/>
@@ -1696,17 +1692,13 @@
       <c r="D21" s="1"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="21" t="s">
-        <v>41</v>
-      </c>
+      <c r="A23" s="1"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="21" t="s">
-        <v>46</v>
-      </c>
+      <c r="A24" s="1"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="21"/>
+      <c r="A25" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -1729,21 +1721,21 @@
       <c r="A1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="4">
-        <v>1</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10" t="s">
+      <c r="B1" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10" t="s">
+      <c r="F1" s="16"/>
+      <c r="G1" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="10"/>
+      <c r="H1" s="16"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
@@ -1775,618 +1767,618 @@
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" cm="1">
+      <c r="B3" s="2" t="e" cm="1">
         <f t="array" ref="B3">INDEX(Szenarien!B:S, $B$1+2, 1)</f>
-        <v>50</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C3" s="2">
         <f>Lösungen!B2</f>
-        <v>2</v>
-      </c>
-      <c r="D3" s="2">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="e">
         <f>PRODUCT(B3,C3)</f>
-        <v>100</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E3" s="2">
         <f>Lösungen!C2</f>
-        <v>1</v>
-      </c>
-      <c r="F3" s="2">
+        <v>2</v>
+      </c>
+      <c r="F3" s="2" t="e">
         <f>PRODUCT(B3,E3)</f>
-        <v>50</v>
+        <v>#VALUE!</v>
       </c>
       <c r="G3" s="2">
         <f>Lösungen!D2</f>
         <v>3</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="2" t="e">
         <f>PRODUCT(B3,G3)</f>
-        <v>150</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2" cm="1">
+      <c r="B4" s="2" t="e" cm="1">
         <f t="array" ref="B4">INDEX(Szenarien!B:S, $B$1+2, 2)</f>
-        <v>5</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C4" s="2">
         <f>Lösungen!B3</f>
         <v>3</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="2" t="e">
         <f>PRODUCT(B4,C4)</f>
-        <v>15</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E4" s="2">
         <f>Lösungen!C3</f>
         <v>3</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="2" t="e">
         <f>PRODUCT(B4,E4)</f>
-        <v>15</v>
+        <v>#VALUE!</v>
       </c>
       <c r="G4" s="2">
         <f>Lösungen!D3</f>
         <v>1</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="2" t="e">
         <f>PRODUCT(B4,G4)</f>
-        <v>5</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2" cm="1">
+      <c r="B5" s="2" t="e" cm="1">
         <f t="array" ref="B5">INDEX(Szenarien!B:S, $B$1+2, 3)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C5" s="2">
         <f>Lösungen!B4</f>
         <v>1</v>
       </c>
-      <c r="D5" s="2">
-        <f t="shared" ref="D5:D19" si="0">PRODUCT(B5,C5)</f>
-        <v>0</v>
+      <c r="D5" s="2" t="e">
+        <f t="shared" ref="D5:D17" si="0">PRODUCT(B5,C5)</f>
+        <v>#VALUE!</v>
       </c>
       <c r="E5" s="2">
         <f>Lösungen!C4</f>
         <v>3</v>
       </c>
-      <c r="F5" s="2">
-        <f t="shared" ref="F5:F20" si="1">PRODUCT(B5,E5)</f>
-        <v>0</v>
+      <c r="F5" s="2" t="e">
+        <f t="shared" ref="F5:F17" si="1">PRODUCT(B5,E5)</f>
+        <v>#VALUE!</v>
       </c>
       <c r="G5" s="2">
         <f>Lösungen!D4</f>
         <v>2</v>
       </c>
-      <c r="H5" s="2">
-        <f t="shared" ref="H5:H20" si="2">PRODUCT(B5,G5)</f>
-        <v>0</v>
+      <c r="H5" s="2" t="e">
+        <f t="shared" ref="H5:H17" si="2">PRODUCT(B5,G5)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="2" cm="1">
+      <c r="B6" s="2" t="e" cm="1">
         <f t="array" ref="B6">INDEX(Szenarien!B:S, $B$1+2, 4)</f>
-        <v>10</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C6" s="2">
         <f>Lösungen!B5</f>
         <v>3</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="2" t="e">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E6" s="2">
         <f>Lösungen!C5</f>
         <v>3</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="2" t="e">
         <f t="shared" si="1"/>
-        <v>30</v>
+        <v>#VALUE!</v>
       </c>
       <c r="G6" s="2">
         <f>Lösungen!D5</f>
         <v>3</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="2" t="e">
         <f t="shared" si="2"/>
-        <v>30</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="2" cm="1">
+      <c r="B7" s="2" t="e" cm="1">
         <f t="array" ref="B7">INDEX(Szenarien!B:S, $B$1+2, 5)</f>
-        <v>5</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C7" s="2">
         <f>Lösungen!B6</f>
         <v>3</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="2" t="e">
         <f>PRODUCT(B7,C9)</f>
-        <v>15</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E7" s="2">
         <f>Lösungen!C6</f>
         <v>3</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="2" t="e">
         <f>PRODUCT(B7,E9)</f>
-        <v>10</v>
+        <v>#VALUE!</v>
       </c>
       <c r="G7" s="2">
         <f>Lösungen!D6</f>
         <v>3</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="2" t="e">
         <f>PRODUCT(B7,G9)</f>
-        <v>10</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="2" cm="1">
+      <c r="B8" s="2" t="e" cm="1">
         <f t="array" ref="B8">INDEX(Szenarien!B:S, $B$1+2, 6)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C8" s="2">
         <f>Lösungen!B7</f>
         <v>3</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="2" t="e">
         <f t="shared" ref="D8:D9" si="3">PRODUCT(B8,C8)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E8" s="2">
         <f>Lösungen!C7</f>
         <v>3</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F8" s="2" t="e">
         <f t="shared" ref="F8:F9" si="4">PRODUCT(B8,E8)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="G8" s="2">
         <f>Lösungen!D7</f>
         <v>3</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="2" t="e">
         <f t="shared" ref="H8:H9" si="5">PRODUCT(B8,G8)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="2" cm="1">
+      <c r="B9" s="2" t="e" cm="1">
         <f t="array" ref="B9">INDEX(Szenarien!B:S, $B$1+2, 7)</f>
-        <v>7</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C9" s="2">
         <f>Lösungen!B8</f>
         <v>3</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="2" t="e">
         <f t="shared" si="3"/>
-        <v>21</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E9" s="2">
         <f>Lösungen!C8</f>
         <v>2</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="2" t="e">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>#VALUE!</v>
       </c>
       <c r="G9" s="2">
         <f>Lösungen!D8</f>
         <v>2</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="2" t="e">
         <f t="shared" si="5"/>
-        <v>14</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="2" cm="1">
+      <c r="B10" s="2" t="e" cm="1">
         <f t="array" ref="B10">INDEX(Szenarien!B:S, $B$1+2, 8)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C10" s="2">
         <f>Lösungen!B9</f>
         <v>3</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="2" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E10" s="2">
         <f>Lösungen!C9</f>
         <v>3</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F10" s="2" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="G10" s="2">
         <f>Lösungen!D9</f>
         <v>3</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="2" t="e">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="2" cm="1">
+      <c r="B11" s="2" t="e" cm="1">
         <f t="array" ref="B11">INDEX(Szenarien!B:S, $B$1+2, 9)</f>
-        <v>3</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C11" s="2">
         <f>Lösungen!B10</f>
         <v>3</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="2" t="e">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E11" s="2">
         <f>Lösungen!C10</f>
         <v>1</v>
       </c>
-      <c r="F11" s="2">
+      <c r="F11" s="2" t="e">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>#VALUE!</v>
       </c>
       <c r="G11" s="2">
         <f>Lösungen!D10</f>
         <v>1</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="2" t="e">
         <f t="shared" si="2"/>
-        <v>3</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="2" cm="1">
+      <c r="B12" s="2" t="e" cm="1">
         <f t="array" ref="B12">INDEX(Szenarien!B:S, $B$1+2, 10)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C12" s="2">
         <f>Lösungen!B11</f>
         <v>3</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="2" t="e">
         <f t="shared" ref="D12" si="6">PRODUCT(B12,C16)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E12" s="2">
         <f>Lösungen!C11</f>
         <v>2</v>
       </c>
-      <c r="F12" s="2">
+      <c r="F12" s="2" t="e">
         <f t="shared" ref="F12" si="7">PRODUCT(B12,E16)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="G12" s="2">
         <f>Lösungen!D11</f>
         <v>1</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="2" t="e">
         <f t="shared" ref="H12" si="8">PRODUCT(B12,G16)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B13" s="2" cm="1">
+        <v>49</v>
+      </c>
+      <c r="B13" s="2" t="e" cm="1">
         <f t="array" ref="B13">INDEX(Szenarien!B:S, $B$1+2, 11)</f>
-        <v>2.5</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C13" s="2">
         <f>Lösungen!B12</f>
         <v>3</v>
       </c>
-      <c r="D13" s="2">
-        <f t="shared" ref="D13:D16" si="9">PRODUCT(B13,C13)</f>
-        <v>7.5</v>
+      <c r="D13" s="2" t="e">
+        <f t="shared" ref="D13" si="9">PRODUCT(B13,C13)</f>
+        <v>#VALUE!</v>
       </c>
       <c r="E13" s="2">
         <f>Lösungen!C12</f>
         <v>3</v>
       </c>
-      <c r="F13" s="2">
-        <f t="shared" ref="F13:F16" si="10">PRODUCT(B13,E13)</f>
-        <v>7.5</v>
+      <c r="F13" s="2" t="e">
+        <f t="shared" ref="F13" si="10">PRODUCT(B13,E13)</f>
+        <v>#VALUE!</v>
       </c>
       <c r="G13" s="2">
         <f>Lösungen!D12</f>
         <v>2</v>
       </c>
-      <c r="H13" s="2">
-        <f t="shared" ref="H13:H16" si="11">PRODUCT(B13,G13)</f>
-        <v>5</v>
+      <c r="H13" s="2" t="e">
+        <f t="shared" ref="H13" si="11">PRODUCT(B13,G13)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B14" s="2" cm="1">
+        <v>45</v>
+      </c>
+      <c r="B14" s="2" t="e" cm="1">
         <f t="array" ref="B14">INDEX(Szenarien!B:S, $B$1+2, 12)</f>
-        <v>2.5</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C14" s="2">
         <f>Lösungen!B13</f>
         <v>3</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="2" t="e">
         <f>PRODUCT(B14,C14)</f>
-        <v>7.5</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E14" s="2">
         <f>Lösungen!C13</f>
         <v>1</v>
       </c>
-      <c r="F14" s="2">
+      <c r="F14" s="2" t="e">
         <f>PRODUCT(B14,E14)</f>
-        <v>2.5</v>
+        <v>#VALUE!</v>
       </c>
       <c r="G14" s="2">
         <f>Lösungen!D13</f>
         <v>1</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="2" t="e">
         <f>PRODUCT(B14,G14)</f>
-        <v>2.5</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="2" cm="1">
+      <c r="B15" s="2" t="e" cm="1">
         <f t="array" ref="B15">INDEX(Szenarien!B:S, $B$1+2, 13)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C15" s="2">
         <f>Lösungen!B14</f>
         <v>3</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="2" t="e">
         <f>PRODUCT(B15,C15)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E15" s="2">
         <f>Lösungen!C14</f>
         <v>3</v>
       </c>
-      <c r="F15" s="2">
+      <c r="F15" s="2" t="e">
         <f>PRODUCT(B15,E15)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="G15" s="2">
         <f>Lösungen!D14</f>
         <v>3</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="2" t="e">
         <f>PRODUCT(B15,G15)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B16" s="2" cm="1">
+      <c r="B16" s="2" t="e" cm="1">
         <f t="array" ref="B16">INDEX(Szenarien!B:S, $B$1+2, 14)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C16" s="2">
         <f>Lösungen!B15</f>
         <v>3</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="2" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E16" s="2">
         <f>Lösungen!C15</f>
         <v>3</v>
       </c>
-      <c r="F16" s="2">
+      <c r="F16" s="2" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="G16" s="2">
         <f>Lösungen!D15</f>
         <v>1</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="2" t="e">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B17" s="2" cm="1">
+      <c r="B17" s="2" t="e" cm="1">
         <f t="array" ref="B17">INDEX(Szenarien!B:S, $B$1+2, 15)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C17" s="2">
         <f>Lösungen!B16</f>
         <v>2</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="2" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E17" s="2">
         <f>Lösungen!C16</f>
         <v>3</v>
       </c>
-      <c r="F17" s="2">
+      <c r="F17" s="2" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="G17" s="2">
         <f>Lösungen!D16</f>
         <v>1</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="2" t="e">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B18" s="2" cm="1">
+      <c r="B18" s="2" t="e" cm="1">
         <f t="array" ref="B18">INDEX(Szenarien!B:S, $B$1+2, 16)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C18" s="2">
         <f>Lösungen!B17</f>
         <v>1</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="2" t="e">
         <f>PRODUCT(B18,C20)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E18" s="2">
         <f>Lösungen!C17</f>
         <v>3</v>
       </c>
-      <c r="F18" s="2">
+      <c r="F18" s="2" t="e">
         <f>PRODUCT(B18,E20)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="G18" s="2">
         <f>Lösungen!D17</f>
         <v>1</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="2" t="e">
         <f>PRODUCT(B18,G20)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B19" s="2" cm="1">
+      <c r="B19" s="2" t="e" cm="1">
         <f t="array" ref="B19">INDEX(Szenarien!B:S, $B$1+2, 17)</f>
-        <v>10</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C19" s="2">
         <f>Lösungen!B18</f>
         <v>3</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="2" t="e">
         <f t="shared" ref="D19:D20" si="12">PRODUCT(B19,C19)</f>
-        <v>30</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E19" s="2">
         <f>Lösungen!C18</f>
         <v>1</v>
       </c>
-      <c r="F19" s="2">
+      <c r="F19" s="2" t="e">
         <f t="shared" ref="F19:F20" si="13">PRODUCT(B19,E19)</f>
-        <v>10</v>
+        <v>#VALUE!</v>
       </c>
       <c r="G19" s="2">
         <f>Lösungen!D18</f>
         <v>2</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="2" t="e">
         <f t="shared" ref="H19:H20" si="14">PRODUCT(B19,G19)</f>
-        <v>20</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="2" cm="1">
+      <c r="B20" s="2" t="e" cm="1">
         <f t="array" ref="B20">INDEX(Szenarien!B:S, $B$1+2, 18)</f>
-        <v>5</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C20" s="2">
         <f>Lösungen!B19</f>
         <v>3</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="2" t="e">
         <f t="shared" si="12"/>
-        <v>15</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E20" s="2">
         <f>Lösungen!C19</f>
         <v>1</v>
       </c>
-      <c r="F20" s="2">
+      <c r="F20" s="2" t="e">
         <f t="shared" si="13"/>
-        <v>5</v>
+        <v>#VALUE!</v>
       </c>
       <c r="G20" s="2">
         <f>Lösungen!D19</f>
         <v>2</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="2" t="e">
         <f t="shared" si="14"/>
-        <v>10</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B21" s="5">
+      <c r="B21" s="5" t="e">
         <f>SUM(B3:B20)</f>
-        <v>100</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C21" s="5"/>
-      <c r="D21" s="5">
+      <c r="D21" s="5" t="e">
         <f>SUM(D3:D20)</f>
-        <v>250</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E21" s="5"/>
-      <c r="F21" s="5">
+      <c r="F21" s="5" t="e">
         <f>SUM(F3:F20)</f>
-        <v>147</v>
+        <v>#VALUE!</v>
       </c>
       <c r="G21" s="5"/>
-      <c r="H21" s="5">
-        <f t="shared" ref="D21:H21" si="15">SUM(H3:H20)</f>
-        <v>249.5</v>
+      <c r="H21" s="5" t="e">
+        <f t="shared" ref="H21" si="15">SUM(H3:H20)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -2395,11 +2387,20 @@
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
+      <c r="D22" s="5" t="e">
+        <f>1+(F21&gt;D21)+(H21&gt;D21)</f>
+        <v>#VALUE!</v>
+      </c>
       <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
+      <c r="F22" s="5" t="e">
+        <f>1+(D21&gt;F21)+(H21&gt;F21)</f>
+        <v>#VALUE!</v>
+      </c>
       <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
+      <c r="H22" s="5" t="e">
+        <f>1+(D21&gt;H21)+(F21&gt;H21)</f>
+        <v>#VALUE!</v>
+      </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
@@ -2440,18 +2441,18 @@
       <c r="B1" s="4">
         <v>1</v>
       </c>
-      <c r="C1" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10" t="s">
+      <c r="C1" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10" t="s">
+      <c r="F1" s="16"/>
+      <c r="G1" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="10"/>
+      <c r="H1" s="16"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
@@ -2489,19 +2490,19 @@
       </c>
       <c r="C3" s="2">
         <f>Lösungen!B2</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" s="2">
         <f>PRODUCT(B3,C3)</f>
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E3" s="2">
         <f>Lösungen!C2</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" s="2">
         <f>PRODUCT(B3,E3)</f>
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="G3" s="2">
         <f>Lösungen!D2</f>
@@ -2558,7 +2559,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="2">
-        <f t="shared" ref="D5:D19" si="0">PRODUCT(B5,C5)</f>
+        <f t="shared" ref="D5:D6" si="0">PRODUCT(B5,C5)</f>
         <v>0</v>
       </c>
       <c r="E5" s="2">
@@ -2566,7 +2567,7 @@
         <v>3</v>
       </c>
       <c r="F5" s="2">
-        <f t="shared" ref="F5:F20" si="1">PRODUCT(B5,E5)</f>
+        <f t="shared" ref="F5:F6" si="1">PRODUCT(B5,E5)</f>
         <v>0</v>
       </c>
       <c r="G5" s="2">
@@ -2574,7 +2575,7 @@
         <v>2</v>
       </c>
       <c r="H5" s="2">
-        <f t="shared" ref="H5:H20" si="2">PRODUCT(B5,G5)</f>
+        <f t="shared" ref="H5:H6" si="2">PRODUCT(B5,G5)</f>
         <v>0</v>
       </c>
     </row>
@@ -2811,7 +2812,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B13" s="2" cm="1">
         <f t="array" ref="B13">INDEX(Szenarien!B:S, $B$1+2, 11)</f>
@@ -2844,7 +2845,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B14" s="2" cm="1">
         <f t="array" ref="B14">INDEX(Szenarien!B:S, $B$1+2, 12)</f>
@@ -2921,7 +2922,7 @@
         <v>3</v>
       </c>
       <c r="D16" s="2">
-        <f t="shared" ref="D16:D30" si="12">PRODUCT(B16,C16)</f>
+        <f t="shared" ref="D16:D17" si="12">PRODUCT(B16,C16)</f>
         <v>0</v>
       </c>
       <c r="E16" s="2">
@@ -2929,7 +2930,7 @@
         <v>3</v>
       </c>
       <c r="F16" s="2">
-        <f t="shared" ref="F16:F31" si="13">PRODUCT(B16,E16)</f>
+        <f t="shared" ref="F16:F17" si="13">PRODUCT(B16,E16)</f>
         <v>0</v>
       </c>
       <c r="G16" s="2">
@@ -2937,7 +2938,7 @@
         <v>1</v>
       </c>
       <c r="H16" s="2">
-        <f t="shared" ref="H16:H31" si="14">PRODUCT(B16,G16)</f>
+        <f t="shared" ref="H16:H17" si="14">PRODUCT(B16,G16)</f>
         <v>0</v>
       </c>
     </row>
@@ -3084,16 +3085,16 @@
       <c r="C21" s="5"/>
       <c r="D21" s="5">
         <f>SUM(D3:D20)</f>
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="E21" s="5"/>
       <c r="F21" s="5">
         <f>SUM(F3:F20)</f>
-        <v>147</v>
+        <v>197</v>
       </c>
       <c r="G21" s="5"/>
       <c r="H21" s="5">
-        <f t="shared" ref="H21:L21" si="18">SUM(H3:H20)</f>
+        <f t="shared" ref="H21" si="18">SUM(H3:H20)</f>
         <v>249.5</v>
       </c>
     </row>
@@ -3103,11 +3104,20 @@
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
+      <c r="D22" s="5">
+        <f>1+(F21&gt;D21)+(H21&gt;D21)</f>
+        <v>2</v>
+      </c>
       <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
+      <c r="F22" s="5">
+        <f>1+(D21&gt;F21)+(H21&gt;F21)</f>
+        <v>3</v>
+      </c>
       <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
+      <c r="H22" s="5">
+        <f>1+(D21&gt;H21)+(F21&gt;H21)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
@@ -3148,18 +3158,18 @@
       <c r="B1" s="4">
         <v>2</v>
       </c>
-      <c r="C1" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10" t="s">
+      <c r="C1" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10" t="s">
+      <c r="F1" s="16"/>
+      <c r="G1" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="10"/>
+      <c r="H1" s="16"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
@@ -3197,19 +3207,19 @@
       </c>
       <c r="C3" s="2">
         <f>Lösungen!B2</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" s="2">
         <f>PRODUCT(B3,C3)</f>
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="E3" s="2">
         <f>Lösungen!C2</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" s="2">
         <f>PRODUCT(B3,E3)</f>
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="G3" s="2">
         <f>Lösungen!D2</f>
@@ -3266,7 +3276,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="2">
-        <f t="shared" ref="D5:D19" si="0">PRODUCT(B5,C5)</f>
+        <f t="shared" ref="D5:D6" si="0">PRODUCT(B5,C5)</f>
         <v>15</v>
       </c>
       <c r="E5" s="2">
@@ -3274,7 +3284,7 @@
         <v>3</v>
       </c>
       <c r="F5" s="2">
-        <f t="shared" ref="F5:F20" si="1">PRODUCT(B5,E5)</f>
+        <f t="shared" ref="F5:F6" si="1">PRODUCT(B5,E5)</f>
         <v>45</v>
       </c>
       <c r="G5" s="2">
@@ -3282,7 +3292,7 @@
         <v>2</v>
       </c>
       <c r="H5" s="2">
-        <f t="shared" ref="H5:H20" si="2">PRODUCT(B5,G5)</f>
+        <f t="shared" ref="H5:H6" si="2">PRODUCT(B5,G5)</f>
         <v>30</v>
       </c>
     </row>
@@ -3519,7 +3529,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B13" s="2" cm="1">
         <f t="array" ref="B13">INDEX(Szenarien!B:S, $B$1+2, 11)</f>
@@ -3552,7 +3562,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B14" s="2" cm="1">
         <f t="array" ref="B14">INDEX(Szenarien!B:S, $B$1+2, 12)</f>
@@ -3629,7 +3639,7 @@
         <v>3</v>
       </c>
       <c r="D16" s="2">
-        <f t="shared" ref="D16:D30" si="12">PRODUCT(B16,C16)</f>
+        <f t="shared" ref="D16:D17" si="12">PRODUCT(B16,C16)</f>
         <v>0</v>
       </c>
       <c r="E16" s="2">
@@ -3637,7 +3647,7 @@
         <v>3</v>
       </c>
       <c r="F16" s="2">
-        <f t="shared" ref="F16:F31" si="13">PRODUCT(B16,E16)</f>
+        <f t="shared" ref="F16:F17" si="13">PRODUCT(B16,E16)</f>
         <v>0</v>
       </c>
       <c r="G16" s="2">
@@ -3645,7 +3655,7 @@
         <v>1</v>
       </c>
       <c r="H16" s="2">
-        <f t="shared" ref="H16:H31" si="14">PRODUCT(B16,G16)</f>
+        <f t="shared" ref="H16:H17" si="14">PRODUCT(B16,G16)</f>
         <v>0</v>
       </c>
     </row>
@@ -3792,16 +3802,16 @@
       <c r="C21" s="5"/>
       <c r="D21" s="5">
         <f>SUM(D3:D20)</f>
-        <v>255</v>
+        <v>240</v>
       </c>
       <c r="E21" s="5"/>
       <c r="F21" s="5">
         <f>SUM(F3:F20)</f>
-        <v>210</v>
+        <v>225</v>
       </c>
       <c r="G21" s="5"/>
       <c r="H21" s="5">
-        <f t="shared" ref="H21:L21" si="18">SUM(H3:H20)</f>
+        <f t="shared" ref="H21" si="18">SUM(H3:H20)</f>
         <v>192.5</v>
       </c>
     </row>
@@ -3811,11 +3821,20 @@
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
+      <c r="D22" s="5">
+        <f>1+(F21&gt;D21)+(H21&gt;D21)</f>
+        <v>1</v>
+      </c>
       <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
+      <c r="F22" s="5">
+        <f>1+(D21&gt;F21)+(H21&gt;F21)</f>
+        <v>2</v>
+      </c>
       <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
+      <c r="H22" s="5">
+        <f>1+(D21&gt;H21)+(F21&gt;H21)</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
@@ -3856,18 +3875,18 @@
       <c r="B1" s="4">
         <v>3</v>
       </c>
-      <c r="C1" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10" t="s">
+      <c r="C1" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10" t="s">
+      <c r="F1" s="16"/>
+      <c r="G1" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="10"/>
+      <c r="H1" s="16"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
@@ -3905,19 +3924,19 @@
       </c>
       <c r="C3" s="2">
         <f>Lösungen!B2</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" s="2">
         <f>PRODUCT(B3,C3)</f>
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="E3" s="2">
         <f>Lösungen!C2</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" s="2">
         <f>PRODUCT(B3,E3)</f>
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="G3" s="2">
         <f>Lösungen!D2</f>
@@ -3974,7 +3993,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="2">
-        <f t="shared" ref="D5:D19" si="0">PRODUCT(B5,C5)</f>
+        <f t="shared" ref="D5:D6" si="0">PRODUCT(B5,C5)</f>
         <v>15</v>
       </c>
       <c r="E5" s="2">
@@ -3982,7 +4001,7 @@
         <v>3</v>
       </c>
       <c r="F5" s="2">
-        <f t="shared" ref="F5:F20" si="1">PRODUCT(B5,E5)</f>
+        <f t="shared" ref="F5:F6" si="1">PRODUCT(B5,E5)</f>
         <v>45</v>
       </c>
       <c r="G5" s="2">
@@ -3990,7 +4009,7 @@
         <v>2</v>
       </c>
       <c r="H5" s="2">
-        <f t="shared" ref="H5:H20" si="2">PRODUCT(B5,G5)</f>
+        <f t="shared" ref="H5:H6" si="2">PRODUCT(B5,G5)</f>
         <v>30</v>
       </c>
     </row>
@@ -4227,7 +4246,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B13" s="2" cm="1">
         <f t="array" ref="B13">INDEX(Szenarien!B:S, $B$1+2, 11)</f>
@@ -4260,7 +4279,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B14" s="2" cm="1">
         <f t="array" ref="B14">INDEX(Szenarien!B:S, $B$1+2, 12)</f>
@@ -4337,7 +4356,7 @@
         <v>3</v>
       </c>
       <c r="D16" s="2">
-        <f t="shared" ref="D16:D30" si="12">PRODUCT(B16,C16)</f>
+        <f t="shared" ref="D16:D17" si="12">PRODUCT(B16,C16)</f>
         <v>0</v>
       </c>
       <c r="E16" s="2">
@@ -4345,7 +4364,7 @@
         <v>3</v>
       </c>
       <c r="F16" s="2">
-        <f t="shared" ref="F16:F31" si="13">PRODUCT(B16,E16)</f>
+        <f t="shared" ref="F16:F17" si="13">PRODUCT(B16,E16)</f>
         <v>0</v>
       </c>
       <c r="G16" s="2">
@@ -4353,7 +4372,7 @@
         <v>1</v>
       </c>
       <c r="H16" s="2">
-        <f t="shared" ref="H16:H31" si="14">PRODUCT(B16,G16)</f>
+        <f t="shared" ref="H16:H17" si="14">PRODUCT(B16,G16)</f>
         <v>0</v>
       </c>
     </row>
@@ -4500,16 +4519,16 @@
       <c r="C21" s="5"/>
       <c r="D21" s="5">
         <f>SUM(D3:D20)</f>
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="E21" s="5"/>
       <c r="F21" s="5">
         <f>SUM(F3:F20)</f>
-        <v>195</v>
+        <v>210</v>
       </c>
       <c r="G21" s="5"/>
       <c r="H21" s="5">
-        <f t="shared" ref="H21:L21" si="18">SUM(H3:H20)</f>
+        <f t="shared" ref="H21" si="18">SUM(H3:H20)</f>
         <v>190</v>
       </c>
     </row>
@@ -4519,11 +4538,20 @@
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
+      <c r="D22" s="5">
+        <f>1+(F21&gt;D21)+(H21&gt;D21)</f>
+        <v>1</v>
+      </c>
       <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
+      <c r="F22" s="5">
+        <f>1+(D21&gt;F21)+(H21&gt;F21)</f>
+        <v>2</v>
+      </c>
       <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
+      <c r="H22" s="5">
+        <f>1+(D21&gt;H21)+(F21&gt;H21)</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
@@ -4564,18 +4592,18 @@
       <c r="B1" s="4">
         <v>4</v>
       </c>
-      <c r="C1" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10" t="s">
+      <c r="C1" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10" t="s">
+      <c r="F1" s="16"/>
+      <c r="G1" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="10"/>
+      <c r="H1" s="16"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
@@ -4613,19 +4641,19 @@
       </c>
       <c r="C3" s="2">
         <f>Lösungen!B2</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" s="2">
         <f>PRODUCT(B3,C3)</f>
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E3" s="2">
         <f>Lösungen!C2</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" s="2">
         <f>PRODUCT(B3,E3)</f>
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G3" s="2">
         <f>Lösungen!D2</f>
@@ -4682,7 +4710,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="2">
-        <f t="shared" ref="D5:D19" si="0">PRODUCT(B5,C5)</f>
+        <f t="shared" ref="D5:D6" si="0">PRODUCT(B5,C5)</f>
         <v>10</v>
       </c>
       <c r="E5" s="2">
@@ -4690,7 +4718,7 @@
         <v>3</v>
       </c>
       <c r="F5" s="2">
-        <f t="shared" ref="F5:F20" si="1">PRODUCT(B5,E5)</f>
+        <f t="shared" ref="F5:F6" si="1">PRODUCT(B5,E5)</f>
         <v>30</v>
       </c>
       <c r="G5" s="2">
@@ -4698,7 +4726,7 @@
         <v>2</v>
       </c>
       <c r="H5" s="2">
-        <f t="shared" ref="H5:H20" si="2">PRODUCT(B5,G5)</f>
+        <f t="shared" ref="H5:H6" si="2">PRODUCT(B5,G5)</f>
         <v>20</v>
       </c>
     </row>
@@ -4935,7 +4963,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B13" s="2" cm="1">
         <f t="array" ref="B13">INDEX(Szenarien!B:S, $B$1+2, 11)</f>
@@ -4968,7 +4996,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B14" s="2" cm="1">
         <f t="array" ref="B14">INDEX(Szenarien!B:S, $B$1+2, 12)</f>
@@ -5045,7 +5073,7 @@
         <v>3</v>
       </c>
       <c r="D16" s="2">
-        <f t="shared" ref="D16:D30" si="12">PRODUCT(B16,C16)</f>
+        <f t="shared" ref="D16:D17" si="12">PRODUCT(B16,C16)</f>
         <v>30</v>
       </c>
       <c r="E16" s="2">
@@ -5053,7 +5081,7 @@
         <v>3</v>
       </c>
       <c r="F16" s="2">
-        <f t="shared" ref="F16:F31" si="13">PRODUCT(B16,E16)</f>
+        <f t="shared" ref="F16:F17" si="13">PRODUCT(B16,E16)</f>
         <v>30</v>
       </c>
       <c r="G16" s="2">
@@ -5061,7 +5089,7 @@
         <v>1</v>
       </c>
       <c r="H16" s="2">
-        <f t="shared" ref="H16:H31" si="14">PRODUCT(B16,G16)</f>
+        <f t="shared" ref="H16:H17" si="14">PRODUCT(B16,G16)</f>
         <v>10</v>
       </c>
     </row>
@@ -5208,16 +5236,16 @@
       <c r="C21" s="5"/>
       <c r="D21" s="5">
         <f>SUM(D3:D20)</f>
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="E21" s="5"/>
       <c r="F21" s="5">
         <f>SUM(F3:F20)</f>
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="G21" s="5"/>
       <c r="H21" s="5">
-        <f t="shared" ref="H21:L21" si="18">SUM(H3:H20)</f>
+        <f t="shared" ref="H21" si="18">SUM(H3:H20)</f>
         <v>205</v>
       </c>
     </row>
@@ -5227,11 +5255,20 @@
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
+      <c r="D22" s="5">
+        <f>1+(F21&gt;D21)+(H21&gt;D21)</f>
+        <v>1</v>
+      </c>
       <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
+      <c r="F22" s="5">
+        <f>1+(D21&gt;F21)+(H21&gt;F21)</f>
+        <v>2</v>
+      </c>
       <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
+      <c r="H22" s="5">
+        <f>1+(D21&gt;H21)+(F21&gt;H21)</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
@@ -5272,18 +5309,18 @@
       <c r="B1" s="4">
         <v>5</v>
       </c>
-      <c r="C1" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10" t="s">
+      <c r="C1" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10" t="s">
+      <c r="F1" s="16"/>
+      <c r="G1" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="10"/>
+      <c r="H1" s="16"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
@@ -5321,19 +5358,19 @@
       </c>
       <c r="C3" s="2">
         <f>Lösungen!B2</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" s="2">
         <f>PRODUCT(B3,C3)</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E3" s="2">
         <f>Lösungen!C2</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" s="2">
         <f>PRODUCT(B3,E3)</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G3" s="2">
         <f>Lösungen!D2</f>
@@ -5390,7 +5427,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="2">
-        <f t="shared" ref="D5:D19" si="0">PRODUCT(B5,C5)</f>
+        <f t="shared" ref="D5:D6" si="0">PRODUCT(B5,C5)</f>
         <v>10</v>
       </c>
       <c r="E5" s="2">
@@ -5398,7 +5435,7 @@
         <v>3</v>
       </c>
       <c r="F5" s="2">
-        <f t="shared" ref="F5:F20" si="1">PRODUCT(B5,E5)</f>
+        <f t="shared" ref="F5:F6" si="1">PRODUCT(B5,E5)</f>
         <v>30</v>
       </c>
       <c r="G5" s="2">
@@ -5406,7 +5443,7 @@
         <v>2</v>
       </c>
       <c r="H5" s="2">
-        <f t="shared" ref="H5:H20" si="2">PRODUCT(B5,G5)</f>
+        <f t="shared" ref="H5:H6" si="2">PRODUCT(B5,G5)</f>
         <v>20</v>
       </c>
     </row>
@@ -5643,7 +5680,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B13" s="2" cm="1">
         <f t="array" ref="B13">INDEX(Szenarien!B:S, $B$1+2, 11)</f>
@@ -5676,7 +5713,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B14" s="2" cm="1">
         <f t="array" ref="B14">INDEX(Szenarien!B:S, $B$1+2, 12)</f>
@@ -5753,7 +5790,7 @@
         <v>3</v>
       </c>
       <c r="D16" s="2">
-        <f t="shared" ref="D16:D30" si="12">PRODUCT(B16,C16)</f>
+        <f t="shared" ref="D16:D17" si="12">PRODUCT(B16,C16)</f>
         <v>0</v>
       </c>
       <c r="E16" s="2">
@@ -5761,7 +5798,7 @@
         <v>3</v>
       </c>
       <c r="F16" s="2">
-        <f t="shared" ref="F16:F31" si="13">PRODUCT(B16,E16)</f>
+        <f t="shared" ref="F16:F17" si="13">PRODUCT(B16,E16)</f>
         <v>0</v>
       </c>
       <c r="G16" s="2">
@@ -5769,7 +5806,7 @@
         <v>1</v>
       </c>
       <c r="H16" s="2">
-        <f t="shared" ref="H16:H31" si="14">PRODUCT(B16,G16)</f>
+        <f t="shared" ref="H16:H17" si="14">PRODUCT(B16,G16)</f>
         <v>0</v>
       </c>
     </row>
@@ -5916,16 +5953,16 @@
       <c r="C21" s="5"/>
       <c r="D21" s="5">
         <f>SUM(D3:D20)</f>
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="E21" s="5"/>
       <c r="F21" s="5">
         <f>SUM(F3:F20)</f>
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="G21" s="5"/>
       <c r="H21" s="5">
-        <f t="shared" ref="H21:L21" si="18">SUM(H3:H20)</f>
+        <f t="shared" ref="H21" si="18">SUM(H3:H20)</f>
         <v>174</v>
       </c>
     </row>
@@ -5935,11 +5972,20 @@
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
+      <c r="D22" s="5">
+        <f>1+(F21&gt;D21)+(H21&gt;D21)</f>
+        <v>1</v>
+      </c>
       <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
+      <c r="F22" s="5">
+        <f>1+(D21&gt;F21)+(H21&gt;F21)</f>
+        <v>2</v>
+      </c>
       <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
+      <c r="H22" s="5">
+        <f>1+(D21&gt;H21)+(F21&gt;H21)</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
@@ -5980,18 +6026,18 @@
       <c r="B1" s="4">
         <v>6</v>
       </c>
-      <c r="C1" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10" t="s">
+      <c r="C1" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10" t="s">
+      <c r="F1" s="16"/>
+      <c r="G1" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="10"/>
+      <c r="H1" s="16"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
@@ -6029,19 +6075,19 @@
       </c>
       <c r="C3" s="2">
         <f>Lösungen!B2</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" s="2">
         <f>PRODUCT(B3,C3)</f>
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E3" s="2">
         <f>Lösungen!C2</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" s="2">
         <f>PRODUCT(B3,E3)</f>
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G3" s="2">
         <f>Lösungen!D2</f>
@@ -6098,7 +6144,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="2">
-        <f t="shared" ref="D5:D19" si="0">PRODUCT(B5,C5)</f>
+        <f t="shared" ref="D5:D6" si="0">PRODUCT(B5,C5)</f>
         <v>10</v>
       </c>
       <c r="E5" s="2">
@@ -6106,7 +6152,7 @@
         <v>3</v>
       </c>
       <c r="F5" s="2">
-        <f t="shared" ref="F5:F20" si="1">PRODUCT(B5,E5)</f>
+        <f t="shared" ref="F5:F6" si="1">PRODUCT(B5,E5)</f>
         <v>30</v>
       </c>
       <c r="G5" s="2">
@@ -6114,7 +6160,7 @@
         <v>2</v>
       </c>
       <c r="H5" s="2">
-        <f t="shared" ref="H5:H20" si="2">PRODUCT(B5,G5)</f>
+        <f t="shared" ref="H5:H6" si="2">PRODUCT(B5,G5)</f>
         <v>20</v>
       </c>
     </row>
@@ -6351,7 +6397,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B13" s="2" cm="1">
         <f t="array" ref="B13">INDEX(Szenarien!B:S, $B$1+2, 11)</f>
@@ -6384,7 +6430,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B14" s="2" cm="1">
         <f t="array" ref="B14">INDEX(Szenarien!B:S, $B$1+2, 12)</f>
@@ -6461,7 +6507,7 @@
         <v>3</v>
       </c>
       <c r="D16" s="2">
-        <f t="shared" ref="D16:D30" si="12">PRODUCT(B16,C16)</f>
+        <f t="shared" ref="D16:D17" si="12">PRODUCT(B16,C16)</f>
         <v>9.9999999000000006</v>
       </c>
       <c r="E16" s="2">
@@ -6469,7 +6515,7 @@
         <v>3</v>
       </c>
       <c r="F16" s="2">
-        <f t="shared" ref="F16:F31" si="13">PRODUCT(B16,E16)</f>
+        <f t="shared" ref="F16:F17" si="13">PRODUCT(B16,E16)</f>
         <v>9.9999999000000006</v>
       </c>
       <c r="G16" s="2">
@@ -6477,7 +6523,7 @@
         <v>1</v>
       </c>
       <c r="H16" s="2">
-        <f t="shared" ref="H16:H31" si="14">PRODUCT(B16,G16)</f>
+        <f t="shared" ref="H16:H17" si="14">PRODUCT(B16,G16)</f>
         <v>3.3333333000000001</v>
       </c>
     </row>
@@ -6624,16 +6670,16 @@
       <c r="C21" s="5"/>
       <c r="D21" s="5">
         <f>SUM(D3:D20)</f>
-        <v>266.66666550000008</v>
+        <v>256.66666550000008</v>
       </c>
       <c r="E21" s="5"/>
       <c r="F21" s="5">
         <f>SUM(F3:F20)</f>
-        <v>213.33333240000002</v>
+        <v>223.33333240000002</v>
       </c>
       <c r="G21" s="5"/>
       <c r="H21" s="5">
-        <f t="shared" ref="H21:L21" si="18">SUM(H3:H20)</f>
+        <f t="shared" ref="H21" si="18">SUM(H3:H20)</f>
         <v>189.99999920000002</v>
       </c>
     </row>
@@ -6643,11 +6689,20 @@
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
+      <c r="D22" s="5">
+        <f>1+(F21&gt;D21)+(H21&gt;D21)</f>
+        <v>1</v>
+      </c>
       <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
+      <c r="F22" s="5">
+        <f>1+(D21&gt;F21)+(H21&gt;F21)</f>
+        <v>2</v>
+      </c>
       <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
+      <c r="H22" s="5">
+        <f>1+(D21&gt;H21)+(F21&gt;H21)</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>

</xml_diff>